<commit_message>
test(login,registration): update suites, add first-login/pending coverage, device fingerprint helper, /refine skill
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test-case-exports/Login.xlsx
+++ b/test-case-exports/Login.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1370" uniqueCount="241">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1378" uniqueCount="244">
   <si>
     <t>#</t>
   </si>
@@ -483,6 +483,15 @@
     <t>should not display the Log In button when already logged in</t>
   </si>
   <si>
+    <t>BusinessTestCases/Login/functional/LoginOtpAdminConfig.spec.ts</t>
+  </si>
+  <si>
+    <t>Login — Admin OTP Configuration</t>
+  </si>
+  <si>
+    <t>LOGIN OTP operation is locked on (checked and not editable) in the default OTP setting</t>
+  </si>
+  <si>
     <t>BusinessTestCases/Login/functional/LoginOtpFlow.spec.ts</t>
   </si>
   <si>
@@ -708,7 +717,7 @@
     <t>Generated</t>
   </si>
   <si>
-    <t>2026-09-08T15:08:53.422Z</t>
+    <t>2026-09-09T06:44:10.097Z</t>
   </si>
   <si>
     <t>Total test cases</t>
@@ -1137,7 +1146,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I168"/>
+  <dimension ref="A1:I169"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -4262,16 +4271,16 @@
         <v>9</v>
       </c>
       <c r="C108" s="2" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="D108" s="2" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="E108" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F108" s="2" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="G108" s="2" t="s">
         <v>14</v>
@@ -4291,16 +4300,16 @@
         <v>9</v>
       </c>
       <c r="C109" s="2" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="D109" s="2" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="E109" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F109" s="2" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="G109" s="2" t="s">
         <v>14</v>
@@ -4320,16 +4329,16 @@
         <v>9</v>
       </c>
       <c r="C110" s="2" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="D110" s="2" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="E110" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F110" s="2" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="G110" s="2" t="s">
         <v>14</v>
@@ -4349,16 +4358,16 @@
         <v>9</v>
       </c>
       <c r="C111" s="2" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="D111" s="2" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="E111" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F111" s="2" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="G111" s="2" t="s">
         <v>14</v>
@@ -4378,16 +4387,16 @@
         <v>9</v>
       </c>
       <c r="C112" s="2" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="D112" s="2" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="E112" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F112" s="2" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="G112" s="2" t="s">
         <v>14</v>
@@ -4407,16 +4416,16 @@
         <v>9</v>
       </c>
       <c r="C113" s="2" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="D113" s="2" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="E113" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F113" s="2" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="G113" s="2" t="s">
         <v>14</v>
@@ -4436,16 +4445,16 @@
         <v>9</v>
       </c>
       <c r="C114" s="2" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="D114" s="2" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="E114" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F114" s="2" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="G114" s="2" t="s">
         <v>14</v>
@@ -4465,16 +4474,16 @@
         <v>9</v>
       </c>
       <c r="C115" s="2" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="D115" s="2" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="E115" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F115" s="2" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="G115" s="2" t="s">
         <v>14</v>
@@ -4494,16 +4503,16 @@
         <v>9</v>
       </c>
       <c r="C116" s="2" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="D116" s="2" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="E116" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F116" s="2" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="G116" s="2" t="s">
         <v>14</v>
@@ -4523,16 +4532,16 @@
         <v>9</v>
       </c>
       <c r="C117" s="2" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="D117" s="2" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="E117" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F117" s="2" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="G117" s="2" t="s">
         <v>14</v>
@@ -4552,16 +4561,16 @@
         <v>9</v>
       </c>
       <c r="C118" s="2" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="D118" s="2" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="E118" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F118" s="2" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="G118" s="2" t="s">
         <v>14</v>
@@ -4581,16 +4590,16 @@
         <v>9</v>
       </c>
       <c r="C119" s="2" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="D119" s="2" t="s">
-        <v>170</v>
+        <v>160</v>
       </c>
       <c r="E119" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F119" s="2" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="G119" s="2" t="s">
         <v>14</v>
@@ -4610,16 +4619,16 @@
         <v>9</v>
       </c>
       <c r="C120" s="2" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="D120" s="2" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="E120" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F120" s="2" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="G120" s="2" t="s">
         <v>14</v>
@@ -4639,16 +4648,16 @@
         <v>9</v>
       </c>
       <c r="C121" s="2" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="D121" s="2" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="E121" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F121" s="2" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="G121" s="2" t="s">
         <v>14</v>
@@ -4668,16 +4677,16 @@
         <v>9</v>
       </c>
       <c r="C122" s="2" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="D122" s="2" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="E122" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F122" s="2" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="G122" s="2" t="s">
         <v>14</v>
@@ -4697,16 +4706,16 @@
         <v>9</v>
       </c>
       <c r="C123" s="2" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="D123" s="2" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="E123" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F123" s="2" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="G123" s="2" t="s">
         <v>14</v>
@@ -4726,10 +4735,10 @@
         <v>9</v>
       </c>
       <c r="C124" s="2" t="s">
-        <v>176</v>
+        <v>159</v>
       </c>
       <c r="D124" s="2" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="E124" s="2" t="s">
         <v>12</v>
@@ -4755,16 +4764,16 @@
         <v>9</v>
       </c>
       <c r="C125" s="2" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="D125" s="2" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="E125" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F125" s="2" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="G125" s="2" t="s">
         <v>14</v>
@@ -4784,16 +4793,16 @@
         <v>9</v>
       </c>
       <c r="C126" s="2" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="D126" s="2" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="E126" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F126" s="2" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="G126" s="2" t="s">
         <v>14</v>
@@ -4813,16 +4822,16 @@
         <v>9</v>
       </c>
       <c r="C127" s="2" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="D127" s="2" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="E127" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F127" s="2" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="G127" s="2" t="s">
         <v>14</v>
@@ -4842,16 +4851,16 @@
         <v>9</v>
       </c>
       <c r="C128" s="2" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="D128" s="2" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="E128" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F128" s="2" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="G128" s="2" t="s">
         <v>14</v>
@@ -4871,16 +4880,16 @@
         <v>9</v>
       </c>
       <c r="C129" s="2" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="D129" s="2" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="E129" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F129" s="2" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="G129" s="2" t="s">
         <v>14</v>
@@ -4900,10 +4909,10 @@
         <v>9</v>
       </c>
       <c r="C130" s="2" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
       <c r="D130" s="2" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
       <c r="E130" s="2" t="s">
         <v>12</v>
@@ -4929,16 +4938,16 @@
         <v>9</v>
       </c>
       <c r="C131" s="2" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="D131" s="2" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="E131" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F131" s="2" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="G131" s="2" t="s">
         <v>14</v>
@@ -4958,16 +4967,16 @@
         <v>9</v>
       </c>
       <c r="C132" s="2" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="D132" s="2" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="E132" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F132" s="2" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="G132" s="2" t="s">
         <v>14</v>
@@ -4987,16 +4996,16 @@
         <v>9</v>
       </c>
       <c r="C133" s="2" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="D133" s="2" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="E133" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F133" s="2" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="G133" s="2" t="s">
         <v>14</v>
@@ -5016,16 +5025,16 @@
         <v>9</v>
       </c>
       <c r="C134" s="2" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="D134" s="2" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="E134" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F134" s="2" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="G134" s="2" t="s">
         <v>14</v>
@@ -5045,16 +5054,16 @@
         <v>9</v>
       </c>
       <c r="C135" s="2" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="D135" s="2" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="E135" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F135" s="2" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="G135" s="2" t="s">
         <v>14</v>
@@ -5074,16 +5083,16 @@
         <v>9</v>
       </c>
       <c r="C136" s="2" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="D136" s="2" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="E136" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F136" s="2" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="G136" s="2" t="s">
         <v>14</v>
@@ -5103,16 +5112,16 @@
         <v>9</v>
       </c>
       <c r="C137" s="2" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="D137" s="2" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="E137" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F137" s="2" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="G137" s="2" t="s">
         <v>14</v>
@@ -5132,16 +5141,16 @@
         <v>9</v>
       </c>
       <c r="C138" s="2" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="D138" s="2" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="E138" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F138" s="2" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="G138" s="2" t="s">
         <v>14</v>
@@ -5161,16 +5170,16 @@
         <v>9</v>
       </c>
       <c r="C139" s="2" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="D139" s="2" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="E139" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F139" s="2" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="G139" s="2" t="s">
         <v>14</v>
@@ -5190,16 +5199,16 @@
         <v>9</v>
       </c>
       <c r="C140" s="2" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="D140" s="2" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="E140" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F140" s="2" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="G140" s="2" t="s">
         <v>14</v>
@@ -5219,16 +5228,16 @@
         <v>9</v>
       </c>
       <c r="C141" s="2" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="D141" s="2" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="E141" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F141" s="2" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="G141" s="2" t="s">
         <v>14</v>
@@ -5248,16 +5257,16 @@
         <v>9</v>
       </c>
       <c r="C142" s="2" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="D142" s="2" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="E142" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F142" s="2" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="G142" s="2" t="s">
         <v>14</v>
@@ -5277,16 +5286,16 @@
         <v>9</v>
       </c>
       <c r="C143" s="2" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="D143" s="2" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="E143" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F143" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="G143" s="2" t="s">
         <v>14</v>
@@ -5306,16 +5315,16 @@
         <v>9</v>
       </c>
       <c r="C144" s="2" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="D144" s="2" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="E144" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F144" s="2" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="G144" s="2" t="s">
         <v>14</v>
@@ -5335,16 +5344,16 @@
         <v>9</v>
       </c>
       <c r="C145" s="2" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="D145" s="2" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="E145" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F145" s="2" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="G145" s="2" t="s">
         <v>14</v>
@@ -5364,16 +5373,16 @@
         <v>9</v>
       </c>
       <c r="C146" s="2" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="D146" s="2" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="E146" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F146" s="2" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="G146" s="2" t="s">
         <v>14</v>
@@ -5393,16 +5402,16 @@
         <v>9</v>
       </c>
       <c r="C147" s="2" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="D147" s="2" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="E147" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F147" s="2" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="G147" s="2" t="s">
         <v>14</v>
@@ -5422,16 +5431,16 @@
         <v>9</v>
       </c>
       <c r="C148" s="2" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="D148" s="2" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="E148" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F148" s="2" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="G148" s="2" t="s">
         <v>14</v>
@@ -5451,16 +5460,16 @@
         <v>9</v>
       </c>
       <c r="C149" s="2" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="D149" s="2" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="E149" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F149" s="2" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="G149" s="2" t="s">
         <v>14</v>
@@ -5480,16 +5489,16 @@
         <v>9</v>
       </c>
       <c r="C150" s="2" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="D150" s="2" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="E150" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F150" s="2" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="G150" s="2" t="s">
         <v>14</v>
@@ -5509,16 +5518,16 @@
         <v>9</v>
       </c>
       <c r="C151" s="2" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="D151" s="2" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="E151" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F151" s="2" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="G151" s="2" t="s">
         <v>14</v>
@@ -5538,16 +5547,16 @@
         <v>9</v>
       </c>
       <c r="C152" s="2" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="D152" s="2" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="E152" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F152" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="G152" s="2" t="s">
         <v>14</v>
@@ -5567,16 +5576,16 @@
         <v>9</v>
       </c>
       <c r="C153" s="2" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="D153" s="2" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="E153" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F153" s="2" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="G153" s="2" t="s">
         <v>14</v>
@@ -5596,16 +5605,16 @@
         <v>9</v>
       </c>
       <c r="C154" s="2" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="D154" s="2" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="E154" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F154" s="2" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="G154" s="2" t="s">
         <v>14</v>
@@ -5625,16 +5634,16 @@
         <v>9</v>
       </c>
       <c r="C155" s="2" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="D155" s="2" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="E155" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F155" s="2" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="G155" s="2" t="s">
         <v>14</v>
@@ -5654,16 +5663,16 @@
         <v>9</v>
       </c>
       <c r="C156" s="2" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="D156" s="2" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="E156" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F156" s="2" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="G156" s="2" t="s">
         <v>14</v>
@@ -5683,16 +5692,16 @@
         <v>9</v>
       </c>
       <c r="C157" s="2" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="D157" s="2" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="E157" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F157" s="2" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="G157" s="2" t="s">
         <v>14</v>
@@ -5712,16 +5721,16 @@
         <v>9</v>
       </c>
       <c r="C158" s="2" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="D158" s="2" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="E158" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F158" s="2" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="G158" s="2" t="s">
         <v>14</v>
@@ -5741,16 +5750,16 @@
         <v>9</v>
       </c>
       <c r="C159" s="2" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="D159" s="2" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="E159" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F159" s="2" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="G159" s="2" t="s">
         <v>14</v>
@@ -5770,16 +5779,16 @@
         <v>9</v>
       </c>
       <c r="C160" s="2" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="D160" s="2" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="E160" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F160" s="2" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="G160" s="2" t="s">
         <v>14</v>
@@ -5799,16 +5808,16 @@
         <v>9</v>
       </c>
       <c r="C161" s="2" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="D161" s="2" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="E161" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F161" s="2" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="G161" s="2" t="s">
         <v>14</v>
@@ -5828,10 +5837,10 @@
         <v>9</v>
       </c>
       <c r="C162" s="2" t="s">
-        <v>218</v>
+        <v>187</v>
       </c>
       <c r="D162" s="2" t="s">
-        <v>219</v>
+        <v>188</v>
       </c>
       <c r="E162" s="2" t="s">
         <v>12</v>
@@ -5846,7 +5855,7 @@
         <v>15</v>
       </c>
       <c r="I162" s="2" t="s">
-        <v>221</v>
+        <v>12</v>
       </c>
     </row>
     <row r="163" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5857,16 +5866,16 @@
         <v>9</v>
       </c>
       <c r="C163" s="2" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="D163" s="2" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="E163" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F163" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="G163" s="2" t="s">
         <v>14</v>
@@ -5875,7 +5884,7 @@
         <v>15</v>
       </c>
       <c r="I163" s="2" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
     </row>
     <row r="164" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5886,16 +5895,16 @@
         <v>9</v>
       </c>
       <c r="C164" s="2" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="D164" s="2" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="E164" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F164" s="2" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="G164" s="2" t="s">
         <v>14</v>
@@ -5904,7 +5913,7 @@
         <v>15</v>
       </c>
       <c r="I164" s="2" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
     </row>
     <row r="165" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5915,25 +5924,25 @@
         <v>9</v>
       </c>
       <c r="C165" s="2" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="D165" s="2" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="E165" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F165" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="G165" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H165" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I165" s="2" t="s">
         <v>224</v>
-      </c>
-      <c r="G165" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H165" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="I165" s="2" t="s">
-        <v>221</v>
       </c>
     </row>
     <row r="166" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5944,16 +5953,16 @@
         <v>9</v>
       </c>
       <c r="C166" s="2" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="D166" s="2" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="E166" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F166" s="2" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="G166" s="2" t="s">
         <v>14</v>
@@ -5962,7 +5971,7 @@
         <v>15</v>
       </c>
       <c r="I166" s="2" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
     </row>
     <row r="167" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5973,16 +5982,16 @@
         <v>9</v>
       </c>
       <c r="C167" s="2" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="D167" s="2" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="E167" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F167" s="2" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="G167" s="2" t="s">
         <v>14</v>
@@ -5991,7 +6000,7 @@
         <v>15</v>
       </c>
       <c r="I167" s="2" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
     </row>
     <row r="168" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -6002,16 +6011,16 @@
         <v>9</v>
       </c>
       <c r="C168" s="2" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="D168" s="2" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="E168" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F168" s="2" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="G168" s="2" t="s">
         <v>14</v>
@@ -6020,11 +6029,40 @@
         <v>15</v>
       </c>
       <c r="I168" s="2" t="s">
-        <v>228</v>
+        <v>224</v>
+      </c>
+    </row>
+    <row r="169" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A169" s="2">
+        <v>168</v>
+      </c>
+      <c r="B169" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C169" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="D169" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="E169" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F169" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="G169" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H169" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I169" s="2" t="s">
+        <v>231</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I168"/>
+  <autoFilter ref="A1:I169"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -6041,7 +6079,7 @@
   <sheetData>
     <row r="1" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>12</v>
@@ -6057,18 +6095,18 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="B3" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="B4">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -6081,7 +6119,7 @@
     </row>
     <row r="6" spans="1:2" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>12</v>
@@ -6089,7 +6127,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="B7">
         <v>50</v>
@@ -6097,15 +6135,15 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="B8">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="B9">
         <v>39</v>
@@ -6121,7 +6159,7 @@
     </row>
     <row r="11" spans="1:2" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="B11" s="4" t="s">
         <v>12</v>
@@ -6132,7 +6170,7 @@
         <v>14</v>
       </c>
       <c r="B12">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
@@ -6145,7 +6183,7 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="B14">
         <v>0</v>
@@ -6161,7 +6199,7 @@
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="B16">
         <v>13</v>
@@ -6169,10 +6207,10 @@
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="B17">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>